<commit_message>
Table Style: paint rotated text with the font of the table style
A cell in a table with text rotated by 45 degrees got the colour of
Normal, while the rest of the row had the colour of the table style.
DrawRotated, which paints text at angles like that, filled its edit
engine without the font of the table style.

Pass it there too, like the other paint paths do, and fill the edit
engine again when the font of the table style changes between cells.

Change-Id: Ia2a23b6143318a5d896feb0c3f4b75c3c8876a17
Signed-off-by: Balazs Varga <balazs.varga@collabora.com>
Reviewed-on: https://gerrit.collaboraoffice.com/c/online/+/14583
Reviewed-by: Miklos Vajna <vmiklos@collabora.com>
Tested-by: Jenkins CPCI <releng@collaboraoffice.com>
</commit_message>
<xml_diff>
--- a/engine/sc/qa/unit/data/xlsx/tablestyle-cellstyle-excluded-font.xlsx
+++ b/engine/sc/qa/unit/data/xlsx/tablestyle-cellstyle-excluded-font.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\balu\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\bvarga\cp\online\engine\sc\qa\unit\data\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E091B7BE-63A1-4554-9D64-771608FCF0FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C37D447E-11D6-461D-87FD-8EC4445545AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16440" yWindow="2535" windowWidth="28800" windowHeight="15345" xr2:uid="{3F96529C-047B-44F3-973B-513522D9D35B}"/>
+    <workbookView xWindow="11595" yWindow="4125" windowWidth="18900" windowHeight="15345" xr2:uid="{3F96529C-047B-44F3-973B-513522D9D35B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -145,11 +145,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment textRotation="45"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -565,14 +568,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="46.5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4">
         <v>4</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="4">
         <v>41558</v>
       </c>
       <c r="D4">

</xml_diff>